<commit_message>
Fix drivers tab: update June data, add ح/س codes, replace template
</commit_message>
<xml_diff>
--- a/public/templates/timesheet-drivers.xlsx
+++ b/public/templates/timesheet-drivers.xlsx
@@ -1,36 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ihab1980\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E56E8C8-0B4F-44F0-95E0-B1102683FF11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-1545" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1110" yWindow="570" windowWidth="18270" windowHeight="7110"/>
   </bookViews>
   <sheets>
     <sheet name="الفاو " sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="144525"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="Xn3YFQMmgadjBl8vW0I8rAQh3ekCSjPRpSw22WyK+vk="/>
     </ext>
@@ -39,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="48">
   <si>
     <t>رقم العمل : 3432960600</t>
   </si>
@@ -93,6 +73,18 @@
   </si>
   <si>
     <t>A</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>غ</t>
+  </si>
+  <si>
+    <t>ق</t>
   </si>
   <si>
     <t>Q</t>
@@ -164,17 +156,20 @@
     <t>رمز الاجازة المرضية :S</t>
   </si>
   <si>
-    <t xml:space="preserve"> حزيران  لعام 2026</t>
+    <t>م / استمارات ضبط الوقت للسيارات المؤجرة  لشهر حزيران  لعام 2026</t>
   </si>
   <si>
-    <t>م / استمارات ضبط الوقت للسيارات المؤجرة  لشهر</t>
+    <t>س</t>
+  </si>
+  <si>
+    <t>ح</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="25" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -209,6 +204,10 @@
       <u/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -312,21 +311,8 @@
       <family val="2"/>
       <charset val="178"/>
     </font>
-    <font>
-      <b/>
-      <sz val="16"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -363,14 +349,15 @@
         <bgColor rgb="FFF2DBDB"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -431,9 +418,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -462,10 +449,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -474,27 +461,24 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -502,102 +486,100 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
-  <dxfs count="58">
+  <dxfs count="184">
     <dxf>
       <fill>
         <patternFill patternType="lightGray"/>
@@ -605,6 +587,11 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill patternType="gray125"/>
       </fill>
     </dxf>
@@ -625,6 +612,11 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill patternType="gray125"/>
       </fill>
     </dxf>
@@ -645,6 +637,11 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill patternType="gray125"/>
       </fill>
     </dxf>
@@ -665,6 +662,11 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill patternType="gray125"/>
       </fill>
     </dxf>
@@ -685,6 +687,11 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill patternType="gray125"/>
       </fill>
     </dxf>
@@ -705,6 +712,11 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill patternType="gray125"/>
       </fill>
     </dxf>
@@ -725,6 +737,11 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill patternType="gray125"/>
       </fill>
     </dxf>
@@ -745,6 +762,11 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill patternType="gray125"/>
       </fill>
     </dxf>
@@ -765,6 +787,11 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill patternType="gray125"/>
       </fill>
     </dxf>
@@ -776,6 +803,123 @@
     <dxf>
       <fill>
         <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid">
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid">
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
       </fill>
     </dxf>
     <dxf>
@@ -853,27 +997,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid">
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor theme="3" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
@@ -910,17 +1033,151 @@
     <dxf>
       <fill>
         <patternFill patternType="lightGrid">
+          <fgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid">
           <fgColor theme="3" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
+        <patternFill patternType="lightGrid">
+          <fgColor theme="3" tint="0.59996337778862885"/>
+          <bgColor theme="3" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="darkVertical">
+          <fgColor theme="0" tint="-0.14996795556505021"/>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightUp">
+          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="darkHorizontal">
+          <fgColor theme="3" tint="0.59996337778862885"/>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightUp">
+          <fgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightUp">
+          <fgColor theme="5"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="darkTrellis">
+          <fgColor rgb="FFC00000"/>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="lightGrid">
+          <fgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid">
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid">
+          <fgColor theme="3" tint="0.59996337778862885"/>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid">
+          <fgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid">
+          <fgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid">
+          <fgColor theme="3" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill patternType="lightGray"/>
       </fill>
     </dxf>
     <dxf>
       <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill patternType="gray125"/>
       </fill>
     </dxf>
@@ -932,6 +1189,441 @@
     <dxf>
       <fill>
         <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE5B8B7"/>
+          <bgColor rgb="FFE5B8B7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE5B8B7"/>
+          <bgColor rgb="FFE5B8B7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
       </fill>
     </dxf>
   </dxfs>
@@ -939,9 +1631,6 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1144,7 +1833,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AQ1000"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1165,13 +1854,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
@@ -1214,13 +1903,13 @@
       <c r="AQ1" s="7"/>
     </row>
     <row r="2" spans="1:43" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -1309,41 +1998,39 @@
       <c r="AP3" s="8"/>
       <c r="AQ3" s="7"/>
     </row>
-    <row r="4" spans="1:43" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:43" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="7"/>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
-      <c r="F4" s="55" t="s">
-        <v>41</v>
-      </c>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54"/>
-      <c r="J4" s="54"/>
-      <c r="K4" s="54"/>
-      <c r="L4" s="54"/>
-      <c r="M4" s="54"/>
-      <c r="N4" s="53" t="s">
-        <v>42</v>
-      </c>
-      <c r="O4" s="53"/>
-      <c r="P4" s="53"/>
-      <c r="Q4" s="53"/>
-      <c r="R4" s="53"/>
-      <c r="S4" s="53"/>
-      <c r="T4" s="53"/>
-      <c r="U4" s="53"/>
-      <c r="V4" s="53"/>
-      <c r="W4" s="53"/>
-      <c r="X4" s="53"/>
-      <c r="Y4" s="53"/>
-      <c r="Z4" s="53"/>
-      <c r="AA4" s="53"/>
-      <c r="AB4" s="53"/>
-      <c r="AC4" s="53"/>
-      <c r="AD4" s="53"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
+      <c r="M4" s="36"/>
+      <c r="N4" s="36"/>
+      <c r="O4" s="36"/>
+      <c r="P4" s="36"/>
+      <c r="Q4" s="36"/>
+      <c r="R4" s="36"/>
+      <c r="S4" s="36"/>
+      <c r="T4" s="36"/>
+      <c r="U4" s="36"/>
+      <c r="V4" s="36"/>
+      <c r="W4" s="36"/>
+      <c r="X4" s="36"/>
+      <c r="Y4" s="36"/>
+      <c r="Z4" s="36"/>
+      <c r="AA4" s="36"/>
+      <c r="AB4" s="36"/>
+      <c r="AC4" s="36"/>
+      <c r="AD4" s="7"/>
       <c r="AE4" s="7"/>
       <c r="AF4" s="7"/>
       <c r="AG4" s="7"/>
@@ -1404,321 +2091,487 @@
       <c r="AQ5" s="7"/>
     </row>
     <row r="6" spans="1:43" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="39" t="s">
+      <c r="A6" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="40"/>
-      <c r="C6" s="41" t="s">
+      <c r="B6" s="51"/>
+      <c r="C6" s="52" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="42">
+      <c r="D6" s="53">
         <v>1</v>
       </c>
-      <c r="E6" s="42">
+      <c r="E6" s="53">
         <v>2</v>
       </c>
-      <c r="F6" s="42">
+      <c r="F6" s="53">
         <v>3</v>
       </c>
-      <c r="G6" s="42">
+      <c r="G6" s="53">
         <v>4</v>
       </c>
-      <c r="H6" s="42">
+      <c r="H6" s="53">
         <v>5</v>
       </c>
-      <c r="I6" s="42">
+      <c r="I6" s="53">
         <v>6</v>
       </c>
-      <c r="J6" s="42">
+      <c r="J6" s="53">
         <v>7</v>
       </c>
-      <c r="K6" s="42">
+      <c r="K6" s="53">
         <v>8</v>
       </c>
-      <c r="L6" s="42">
+      <c r="L6" s="53">
         <v>9</v>
       </c>
-      <c r="M6" s="42">
+      <c r="M6" s="53">
         <v>10</v>
       </c>
-      <c r="N6" s="42">
+      <c r="N6" s="53">
         <v>11</v>
       </c>
-      <c r="O6" s="42">
+      <c r="O6" s="53">
         <v>12</v>
       </c>
-      <c r="P6" s="42">
+      <c r="P6" s="53">
         <v>13</v>
       </c>
-      <c r="Q6" s="42">
+      <c r="Q6" s="53">
         <v>14</v>
       </c>
-      <c r="R6" s="42">
+      <c r="R6" s="53">
         <v>15</v>
       </c>
-      <c r="S6" s="42">
+      <c r="S6" s="53">
         <v>16</v>
       </c>
-      <c r="T6" s="42">
+      <c r="T6" s="53">
         <v>17</v>
       </c>
-      <c r="U6" s="42">
+      <c r="U6" s="53">
         <v>18</v>
       </c>
-      <c r="V6" s="42">
+      <c r="V6" s="53">
         <v>19</v>
       </c>
-      <c r="W6" s="42">
+      <c r="W6" s="53">
         <v>20</v>
       </c>
-      <c r="X6" s="42">
+      <c r="X6" s="53">
         <v>21</v>
       </c>
-      <c r="Y6" s="42">
+      <c r="Y6" s="53">
         <v>22</v>
       </c>
-      <c r="Z6" s="42">
+      <c r="Z6" s="53">
         <v>23</v>
       </c>
-      <c r="AA6" s="42">
+      <c r="AA6" s="53">
         <v>24</v>
       </c>
-      <c r="AB6" s="42">
+      <c r="AB6" s="53">
         <v>25</v>
       </c>
-      <c r="AC6" s="42">
+      <c r="AC6" s="53">
         <v>26</v>
       </c>
-      <c r="AD6" s="42">
+      <c r="AD6" s="53">
         <v>27</v>
       </c>
-      <c r="AE6" s="42">
+      <c r="AE6" s="53">
         <v>28</v>
       </c>
-      <c r="AF6" s="42">
+      <c r="AF6" s="53">
         <v>29</v>
       </c>
-      <c r="AG6" s="42">
+      <c r="AG6" s="53">
         <v>30</v>
       </c>
-      <c r="AH6" s="41" t="s">
+      <c r="AH6" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="AI6" s="41" t="s">
+      <c r="AI6" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="AJ6" s="39" t="s">
+      <c r="AJ6" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="AK6" s="39" t="s">
+      <c r="AK6" s="50" t="s">
         <v>10</v>
       </c>
-      <c r="AL6" s="43" t="s">
+      <c r="AL6" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="AM6" s="43" t="s">
+      <c r="AM6" s="54" t="s">
         <v>12</v>
       </c>
-      <c r="AN6" s="43" t="s">
+      <c r="AN6" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="AO6" s="43" t="s">
+      <c r="AO6" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="AP6" s="43" t="s">
+      <c r="AP6" s="54" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:43" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="50" t="s">
+      <c r="A7" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="52"/>
-      <c r="C7" s="31" t="s">
+      <c r="B7" s="40"/>
+      <c r="C7" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="37"/>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="38"/>
-      <c r="H7" s="38"/>
-      <c r="I7" s="38"/>
-      <c r="J7" s="37"/>
-      <c r="K7" s="37"/>
-      <c r="L7" s="37"/>
-      <c r="M7" s="37"/>
-      <c r="N7" s="37"/>
-      <c r="O7" s="38"/>
-      <c r="P7" s="38"/>
-      <c r="Q7" s="37"/>
-      <c r="R7" s="37"/>
-      <c r="S7" s="38"/>
-      <c r="T7" s="37"/>
-      <c r="U7" s="37"/>
-      <c r="V7" s="38"/>
-      <c r="W7" s="38"/>
-      <c r="X7" s="37"/>
-      <c r="Y7" s="37"/>
-      <c r="Z7" s="37"/>
-      <c r="AA7" s="37"/>
-      <c r="AB7" s="37"/>
-      <c r="AC7" s="38"/>
-      <c r="AD7" s="38"/>
-      <c r="AE7" s="37"/>
-      <c r="AF7" s="37"/>
-      <c r="AG7" s="37"/>
-      <c r="AH7" s="32"/>
-      <c r="AI7" s="32"/>
-      <c r="AJ7" s="33"/>
-      <c r="AK7" s="33"/>
-      <c r="AL7" s="33"/>
-      <c r="AM7" s="33"/>
-      <c r="AN7" s="33"/>
-      <c r="AO7" s="33"/>
-      <c r="AP7" s="33"/>
+      <c r="D7" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="48"/>
+      <c r="F7" s="48" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="H7" s="49" t="s">
+        <v>18</v>
+      </c>
+      <c r="I7" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="J7" s="48" t="s">
+        <v>21</v>
+      </c>
+      <c r="K7" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="L7" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="M7" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="N7" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="O7" s="49" t="s">
+        <v>18</v>
+      </c>
+      <c r="P7" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q7" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="R7" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="S7" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="T7" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="U7" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="V7" s="49" t="s">
+        <v>18</v>
+      </c>
+      <c r="W7" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="X7" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="Y7" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="Z7" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="AA7" s="48"/>
+      <c r="AB7" s="48"/>
+      <c r="AC7" s="49" t="s">
+        <v>18</v>
+      </c>
+      <c r="AD7" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE7" s="48"/>
+      <c r="AF7" s="48"/>
+      <c r="AG7" s="48"/>
+      <c r="AH7" s="42"/>
+      <c r="AI7" s="42">
+        <f>COUNTIF(D7:AG7,"ف")</f>
+        <v>0</v>
+      </c>
+      <c r="AJ7" s="43">
+        <f>COUNTIF(D7:AG7,"أ")</f>
+        <v>0</v>
+      </c>
+      <c r="AK7" s="43">
+        <f>COUNTIF(D7:AG7,"ب")</f>
+        <v>0</v>
+      </c>
+      <c r="AL7" s="43">
+        <f t="shared" ref="AL7:AL10" si="0">COUNTIF(D7:AH7,"ر")</f>
+        <v>0</v>
+      </c>
+      <c r="AM7" s="43">
+        <f>COUNTIF(D7:AG7,"ق")</f>
+        <v>1</v>
+      </c>
+      <c r="AN7" s="43">
+        <f>COUNTIF(G7:AI7,"Y")</f>
+        <v>6</v>
+      </c>
+      <c r="AO7" s="43"/>
+      <c r="AP7" s="43"/>
       <c r="AQ7" s="10"/>
     </row>
     <row r="8" spans="1:43" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="51"/>
-      <c r="B8" s="51"/>
-      <c r="C8" s="34" t="s">
+      <c r="A8" s="44"/>
+      <c r="B8" s="44"/>
+      <c r="C8" s="45" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="48"/>
+      <c r="E8" s="48"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="49"/>
+      <c r="H8" s="49"/>
+      <c r="I8" s="49"/>
+      <c r="J8" s="48"/>
+      <c r="K8" s="48"/>
+      <c r="L8" s="48"/>
+      <c r="M8" s="48"/>
+      <c r="N8" s="48"/>
+      <c r="O8" s="49"/>
+      <c r="P8" s="49"/>
+      <c r="Q8" s="48"/>
+      <c r="R8" s="48"/>
+      <c r="S8" s="49"/>
+      <c r="T8" s="48"/>
+      <c r="U8" s="48"/>
+      <c r="V8" s="49"/>
+      <c r="W8" s="49"/>
+      <c r="X8" s="48"/>
+      <c r="Y8" s="48"/>
+      <c r="Z8" s="48"/>
+      <c r="AA8" s="48"/>
+      <c r="AB8" s="48"/>
+      <c r="AC8" s="49"/>
+      <c r="AD8" s="49"/>
+      <c r="AE8" s="48"/>
+      <c r="AF8" s="48"/>
+      <c r="AG8" s="48"/>
+      <c r="AH8" s="46">
+        <f>SUM(D8:AG8)</f>
+        <v>0</v>
+      </c>
+      <c r="AI8" s="42">
+        <f>COUNTIF(D8:AG8,"ف")</f>
+        <v>0</v>
+      </c>
+      <c r="AJ8" s="43">
+        <f>COUNTIF(D8:AG8,"أ")</f>
+        <v>0</v>
+      </c>
+      <c r="AK8" s="43">
+        <v>0</v>
+      </c>
+      <c r="AL8" s="43">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AM8" s="43">
+        <v>0</v>
+      </c>
+      <c r="AN8" s="43"/>
+      <c r="AO8" s="43"/>
+      <c r="AP8" s="43"/>
+      <c r="AQ8" s="10"/>
+    </row>
+    <row r="9" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="47"/>
+      <c r="C9" s="41" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="E9" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="F9" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="H9" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="37"/>
-      <c r="E8" s="37"/>
-      <c r="F8" s="37"/>
-      <c r="G8" s="38"/>
-      <c r="H8" s="38"/>
-      <c r="I8" s="38"/>
-      <c r="J8" s="37"/>
-      <c r="K8" s="37"/>
-      <c r="L8" s="37"/>
-      <c r="M8" s="37"/>
-      <c r="N8" s="37"/>
-      <c r="O8" s="38"/>
-      <c r="P8" s="38"/>
-      <c r="Q8" s="37"/>
-      <c r="R8" s="37"/>
-      <c r="S8" s="38"/>
-      <c r="T8" s="37"/>
-      <c r="U8" s="37"/>
-      <c r="V8" s="38"/>
-      <c r="W8" s="38"/>
-      <c r="X8" s="37"/>
-      <c r="Y8" s="37"/>
-      <c r="Z8" s="37"/>
-      <c r="AA8" s="37"/>
-      <c r="AB8" s="37"/>
-      <c r="AC8" s="38"/>
-      <c r="AD8" s="38"/>
-      <c r="AE8" s="37"/>
-      <c r="AF8" s="37"/>
-      <c r="AG8" s="37"/>
-      <c r="AH8" s="35"/>
-      <c r="AI8" s="32"/>
-      <c r="AJ8" s="33"/>
-      <c r="AK8" s="33"/>
-      <c r="AL8" s="33"/>
-      <c r="AM8" s="33"/>
-      <c r="AN8" s="33"/>
-      <c r="AO8" s="33"/>
-      <c r="AP8" s="33"/>
-      <c r="AQ8" s="10"/>
-    </row>
-    <row r="9" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="33" t="s">
+      <c r="I9" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="36"/>
-      <c r="C9" s="31" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="38"/>
-      <c r="H9" s="38"/>
-      <c r="I9" s="38"/>
-      <c r="J9" s="37"/>
-      <c r="K9" s="37"/>
-      <c r="L9" s="37"/>
-      <c r="M9" s="37"/>
-      <c r="N9" s="37"/>
-      <c r="O9" s="38"/>
-      <c r="P9" s="38"/>
-      <c r="Q9" s="37"/>
-      <c r="R9" s="37"/>
-      <c r="S9" s="38"/>
-      <c r="T9" s="37"/>
-      <c r="U9" s="37"/>
-      <c r="V9" s="38"/>
-      <c r="W9" s="38"/>
-      <c r="X9" s="37"/>
-      <c r="Y9" s="37"/>
-      <c r="Z9" s="37"/>
-      <c r="AA9" s="37"/>
-      <c r="AB9" s="37"/>
-      <c r="AC9" s="38"/>
-      <c r="AD9" s="38"/>
-      <c r="AE9" s="37"/>
-      <c r="AF9" s="37"/>
-      <c r="AG9" s="37"/>
-      <c r="AH9" s="32"/>
-      <c r="AI9" s="32"/>
-      <c r="AJ9" s="33"/>
-      <c r="AK9" s="33"/>
-      <c r="AL9" s="33"/>
-      <c r="AM9" s="33"/>
-      <c r="AN9" s="33"/>
-      <c r="AO9" s="33"/>
-      <c r="AP9" s="33"/>
+      <c r="J9" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="K9" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="L9" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="M9" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="N9" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="O9" s="49" t="s">
+        <v>18</v>
+      </c>
+      <c r="P9" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q9" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="R9" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="S9" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="T9" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="U9" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="V9" s="49" t="s">
+        <v>18</v>
+      </c>
+      <c r="W9" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="X9" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y9" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="Z9" s="48" t="s">
+        <v>20</v>
+      </c>
+      <c r="AA9" s="48"/>
+      <c r="AB9" s="48"/>
+      <c r="AC9" s="49" t="s">
+        <v>18</v>
+      </c>
+      <c r="AD9" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="AE9" s="48"/>
+      <c r="AF9" s="48"/>
+      <c r="AG9" s="48"/>
+      <c r="AH9" s="42"/>
+      <c r="AI9" s="42">
+        <f>COUNTIF(D9:AG9,"ف")</f>
+        <v>0</v>
+      </c>
+      <c r="AJ9" s="43">
+        <f>COUNTIF(D9:AG9,"أ")</f>
+        <v>0</v>
+      </c>
+      <c r="AK9" s="43">
+        <f>COUNTIF(D7:AG7,"ب")</f>
+        <v>0</v>
+      </c>
+      <c r="AL9" s="43">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AM9" s="43">
+        <f>COUNTIF(D7:AG7,"ق")</f>
+        <v>1</v>
+      </c>
+      <c r="AN9" s="43"/>
+      <c r="AO9" s="43"/>
+      <c r="AP9" s="43"/>
       <c r="AQ9" s="10"/>
     </row>
     <row r="10" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="36"/>
-      <c r="B10" s="36"/>
-      <c r="C10" s="34" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="37"/>
-      <c r="E10" s="37"/>
-      <c r="F10" s="37"/>
-      <c r="G10" s="38"/>
-      <c r="H10" s="38"/>
-      <c r="I10" s="38"/>
-      <c r="J10" s="37"/>
-      <c r="K10" s="37"/>
-      <c r="L10" s="37"/>
-      <c r="M10" s="37"/>
-      <c r="N10" s="37"/>
-      <c r="O10" s="38"/>
-      <c r="P10" s="38"/>
-      <c r="Q10" s="37"/>
-      <c r="R10" s="37"/>
-      <c r="S10" s="38"/>
-      <c r="T10" s="37"/>
-      <c r="U10" s="37"/>
-      <c r="V10" s="38"/>
-      <c r="W10" s="38"/>
-      <c r="X10" s="37"/>
-      <c r="Y10" s="37"/>
-      <c r="Z10" s="37"/>
-      <c r="AA10" s="37"/>
-      <c r="AB10" s="37"/>
-      <c r="AC10" s="38"/>
-      <c r="AD10" s="38"/>
-      <c r="AE10" s="37"/>
-      <c r="AF10" s="37"/>
-      <c r="AG10" s="37"/>
-      <c r="AH10" s="35"/>
-      <c r="AI10" s="32"/>
-      <c r="AJ10" s="32"/>
-      <c r="AK10" s="32"/>
-      <c r="AL10" s="32"/>
-      <c r="AM10" s="32"/>
-      <c r="AN10" s="32"/>
-      <c r="AO10" s="33"/>
-      <c r="AP10" s="33"/>
+      <c r="A10" s="47"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="45" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="48"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48"/>
+      <c r="G10" s="49"/>
+      <c r="H10" s="49"/>
+      <c r="I10" s="49"/>
+      <c r="J10" s="48"/>
+      <c r="K10" s="48"/>
+      <c r="L10" s="48"/>
+      <c r="M10" s="48"/>
+      <c r="N10" s="48"/>
+      <c r="O10" s="49"/>
+      <c r="P10" s="49"/>
+      <c r="Q10" s="48"/>
+      <c r="R10" s="48"/>
+      <c r="S10" s="49"/>
+      <c r="T10" s="48"/>
+      <c r="U10" s="48"/>
+      <c r="V10" s="49"/>
+      <c r="W10" s="49"/>
+      <c r="X10" s="48"/>
+      <c r="Y10" s="48"/>
+      <c r="Z10" s="48"/>
+      <c r="AA10" s="48"/>
+      <c r="AB10" s="48"/>
+      <c r="AC10" s="49"/>
+      <c r="AD10" s="49"/>
+      <c r="AE10" s="48"/>
+      <c r="AF10" s="48"/>
+      <c r="AG10" s="48"/>
+      <c r="AH10" s="46">
+        <f>SUM(D10:AG10)</f>
+        <v>0</v>
+      </c>
+      <c r="AI10" s="42">
+        <f>COUNTIF(D10:AG10,"ف")</f>
+        <v>0</v>
+      </c>
+      <c r="AJ10" s="42">
+        <f>COUNTIF(D10:AG10,"أ")</f>
+        <v>0</v>
+      </c>
+      <c r="AK10" s="42">
+        <f>COUNTIF(D10:AG10,"ب")</f>
+        <v>0</v>
+      </c>
+      <c r="AL10" s="42">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AM10" s="42">
+        <v>0</v>
+      </c>
+      <c r="AN10" s="42">
+        <v>0</v>
+      </c>
+      <c r="AO10" s="43"/>
+      <c r="AP10" s="43"/>
       <c r="AQ10" s="10"/>
     </row>
     <row r="11" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1772,62 +2625,62 @@
       <c r="AK12" s="12"/>
       <c r="AM12" s="10"/>
       <c r="AP12" s="14" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="AQ12" s="8"/>
     </row>
     <row r="13" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="47" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="45"/>
+      <c r="A13" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="32"/>
       <c r="C13" s="15"/>
       <c r="D13" s="16"/>
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
       <c r="G13" s="16"/>
       <c r="H13" s="15"/>
-      <c r="I13" s="47" t="s">
-        <v>22</v>
-      </c>
-      <c r="J13" s="45"/>
-      <c r="K13" s="45"/>
-      <c r="L13" s="45"/>
-      <c r="M13" s="45"/>
-      <c r="N13" s="45"/>
-      <c r="O13" s="45"/>
-      <c r="P13" s="45"/>
+      <c r="I13" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="J13" s="32"/>
+      <c r="K13" s="32"/>
+      <c r="L13" s="32"/>
+      <c r="M13" s="32"/>
+      <c r="N13" s="32"/>
+      <c r="O13" s="32"/>
+      <c r="P13" s="32"/>
       <c r="Q13" s="16"/>
       <c r="R13" s="16"/>
       <c r="S13" s="16"/>
       <c r="T13" s="16"/>
       <c r="U13" s="16"/>
       <c r="V13" s="16"/>
-      <c r="W13" s="47" t="s">
-        <v>23</v>
-      </c>
-      <c r="X13" s="45"/>
-      <c r="Y13" s="45"/>
-      <c r="Z13" s="45"/>
-      <c r="AA13" s="45"/>
-      <c r="AB13" s="45"/>
+      <c r="W13" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="X13" s="32"/>
+      <c r="Y13" s="32"/>
+      <c r="Z13" s="32"/>
+      <c r="AA13" s="32"/>
+      <c r="AB13" s="32"/>
       <c r="AC13" s="15"/>
       <c r="AD13" s="15"/>
       <c r="AE13" s="15"/>
       <c r="AF13" s="15"/>
       <c r="AG13" s="15"/>
-      <c r="AH13" s="48" t="s">
-        <v>24</v>
-      </c>
-      <c r="AI13" s="45"/>
-      <c r="AJ13" s="45"/>
-      <c r="AK13" s="45"/>
-      <c r="AL13" s="45"/>
-      <c r="AM13" s="45"/>
-      <c r="AN13" s="45"/>
-      <c r="AO13" s="45"/>
+      <c r="AH13" s="33" t="s">
+        <v>28</v>
+      </c>
+      <c r="AI13" s="32"/>
+      <c r="AJ13" s="32"/>
+      <c r="AK13" s="32"/>
+      <c r="AL13" s="32"/>
+      <c r="AM13" s="32"/>
+      <c r="AN13" s="32"/>
+      <c r="AO13" s="32"/>
       <c r="AP13" s="17" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="AQ13" s="8"/>
     </row>
@@ -1874,7 +2727,7 @@
       <c r="AN14" s="8"/>
       <c r="AO14" s="8"/>
       <c r="AP14" s="17" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="AQ14" s="8"/>
     </row>
@@ -1921,7 +2774,7 @@
       <c r="AN15" s="8"/>
       <c r="AO15" s="8"/>
       <c r="AP15" s="17" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="AQ15" s="8"/>
     </row>
@@ -1968,7 +2821,7 @@
       <c r="AN16" s="8"/>
       <c r="AO16" s="8"/>
       <c r="AP16" s="17" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="AQ16" s="8"/>
     </row>
@@ -2015,7 +2868,7 @@
       <c r="AN17" s="8"/>
       <c r="AO17" s="8"/>
       <c r="AP17" s="17" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="AQ17" s="8"/>
     </row>
@@ -2062,64 +2915,64 @@
       <c r="AN18" s="8"/>
       <c r="AO18" s="8"/>
       <c r="AP18" s="24" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="AQ18" s="8"/>
     </row>
     <row r="19" spans="1:43" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="46" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19" s="45"/>
+      <c r="A19" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" s="32"/>
       <c r="C19" s="25"/>
       <c r="D19" s="26"/>
-      <c r="E19" s="46" t="s">
-        <v>32</v>
-      </c>
-      <c r="F19" s="45"/>
-      <c r="G19" s="45"/>
-      <c r="H19" s="45"/>
-      <c r="I19" s="45"/>
-      <c r="J19" s="45"/>
-      <c r="K19" s="45"/>
-      <c r="L19" s="45"/>
+      <c r="E19" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="F19" s="32"/>
+      <c r="G19" s="32"/>
+      <c r="H19" s="32"/>
+      <c r="I19" s="32"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="32"/>
+      <c r="L19" s="32"/>
       <c r="M19" s="27"/>
       <c r="N19" s="26"/>
       <c r="O19" s="26"/>
-      <c r="P19" s="46" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q19" s="45"/>
-      <c r="R19" s="45"/>
-      <c r="S19" s="45"/>
-      <c r="T19" s="45"/>
-      <c r="U19" s="45"/>
-      <c r="V19" s="45"/>
-      <c r="W19" s="45"/>
-      <c r="X19" s="45"/>
-      <c r="Y19" s="45"/>
+      <c r="P19" s="37" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q19" s="32"/>
+      <c r="R19" s="32"/>
+      <c r="S19" s="32"/>
+      <c r="T19" s="32"/>
+      <c r="U19" s="32"/>
+      <c r="V19" s="32"/>
+      <c r="W19" s="32"/>
+      <c r="X19" s="32"/>
+      <c r="Y19" s="32"/>
       <c r="Z19" s="26"/>
       <c r="AA19" s="26"/>
       <c r="AB19" s="26"/>
       <c r="AC19" s="25"/>
-      <c r="AD19" s="46" t="s">
-        <v>34</v>
-      </c>
-      <c r="AE19" s="45"/>
-      <c r="AF19" s="45"/>
-      <c r="AG19" s="45"/>
-      <c r="AH19" s="45"/>
+      <c r="AD19" s="37" t="s">
+        <v>38</v>
+      </c>
+      <c r="AE19" s="32"/>
+      <c r="AF19" s="32"/>
+      <c r="AG19" s="32"/>
+      <c r="AH19" s="32"/>
       <c r="AI19" s="26"/>
       <c r="AJ19" s="11"/>
       <c r="AK19" s="11"/>
-      <c r="AL19" s="46" t="s">
-        <v>35</v>
-      </c>
-      <c r="AM19" s="45"/>
-      <c r="AN19" s="45"/>
-      <c r="AO19" s="45"/>
+      <c r="AL19" s="37" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM19" s="32"/>
+      <c r="AN19" s="32"/>
+      <c r="AO19" s="32"/>
       <c r="AP19" s="24" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="AQ19" s="8"/>
     </row>
@@ -2129,46 +2982,46 @@
       <c r="C20" s="26"/>
       <c r="D20" s="26"/>
       <c r="E20" s="26"/>
-      <c r="F20" s="44"/>
-      <c r="G20" s="45"/>
-      <c r="H20" s="45"/>
-      <c r="I20" s="45"/>
-      <c r="J20" s="45"/>
-      <c r="K20" s="45"/>
+      <c r="F20" s="38"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="32"/>
+      <c r="K20" s="32"/>
       <c r="L20" s="26"/>
       <c r="M20" s="27"/>
       <c r="N20" s="26"/>
       <c r="O20" s="26"/>
-      <c r="P20" s="44"/>
-      <c r="Q20" s="45"/>
-      <c r="R20" s="45"/>
-      <c r="S20" s="45"/>
-      <c r="T20" s="45"/>
-      <c r="U20" s="45"/>
-      <c r="V20" s="45"/>
-      <c r="W20" s="45"/>
+      <c r="P20" s="38"/>
+      <c r="Q20" s="32"/>
+      <c r="R20" s="32"/>
+      <c r="S20" s="32"/>
+      <c r="T20" s="32"/>
+      <c r="U20" s="32"/>
+      <c r="V20" s="32"/>
+      <c r="W20" s="32"/>
       <c r="X20" s="26"/>
       <c r="Y20" s="26"/>
       <c r="Z20" s="26"/>
       <c r="AA20" s="26"/>
       <c r="AB20" s="26"/>
-      <c r="AC20" s="46" t="s">
-        <v>37</v>
-      </c>
-      <c r="AD20" s="45"/>
-      <c r="AE20" s="45"/>
-      <c r="AF20" s="45"/>
-      <c r="AG20" s="45"/>
-      <c r="AH20" s="45"/>
+      <c r="AC20" s="37" t="s">
+        <v>41</v>
+      </c>
+      <c r="AD20" s="32"/>
+      <c r="AE20" s="32"/>
+      <c r="AF20" s="32"/>
+      <c r="AG20" s="32"/>
+      <c r="AH20" s="32"/>
       <c r="AI20" s="26"/>
       <c r="AJ20" s="11"/>
       <c r="AK20" s="11"/>
-      <c r="AL20" s="46" t="s">
-        <v>38</v>
-      </c>
-      <c r="AM20" s="45"/>
-      <c r="AN20" s="45"/>
-      <c r="AO20" s="45"/>
+      <c r="AL20" s="37" t="s">
+        <v>42</v>
+      </c>
+      <c r="AM20" s="32"/>
+      <c r="AN20" s="32"/>
+      <c r="AO20" s="32"/>
       <c r="AP20" s="8"/>
       <c r="AQ20" s="8"/>
     </row>
@@ -2178,46 +3031,46 @@
       <c r="C21" s="26"/>
       <c r="D21" s="26"/>
       <c r="E21" s="26"/>
-      <c r="F21" s="44"/>
-      <c r="G21" s="45"/>
-      <c r="H21" s="45"/>
-      <c r="I21" s="45"/>
-      <c r="J21" s="45"/>
-      <c r="K21" s="45"/>
+      <c r="F21" s="38"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="32"/>
+      <c r="I21" s="32"/>
+      <c r="J21" s="32"/>
+      <c r="K21" s="32"/>
       <c r="L21" s="26"/>
       <c r="M21" s="27"/>
       <c r="N21" s="26"/>
       <c r="O21" s="26"/>
-      <c r="P21" s="44"/>
-      <c r="Q21" s="45"/>
-      <c r="R21" s="45"/>
-      <c r="S21" s="45"/>
-      <c r="T21" s="45"/>
-      <c r="U21" s="45"/>
-      <c r="V21" s="45"/>
-      <c r="W21" s="45"/>
+      <c r="P21" s="38"/>
+      <c r="Q21" s="32"/>
+      <c r="R21" s="32"/>
+      <c r="S21" s="32"/>
+      <c r="T21" s="32"/>
+      <c r="U21" s="32"/>
+      <c r="V21" s="32"/>
+      <c r="W21" s="32"/>
       <c r="X21" s="26"/>
       <c r="Y21" s="26"/>
       <c r="Z21" s="26"/>
       <c r="AA21" s="26"/>
       <c r="AB21" s="26"/>
-      <c r="AC21" s="46" t="s">
-        <v>39</v>
-      </c>
-      <c r="AD21" s="45"/>
-      <c r="AE21" s="45"/>
-      <c r="AF21" s="45"/>
-      <c r="AG21" s="45"/>
-      <c r="AH21" s="45"/>
+      <c r="AC21" s="37" t="s">
+        <v>43</v>
+      </c>
+      <c r="AD21" s="32"/>
+      <c r="AE21" s="32"/>
+      <c r="AF21" s="32"/>
+      <c r="AG21" s="32"/>
+      <c r="AH21" s="32"/>
       <c r="AI21" s="26"/>
       <c r="AJ21" s="11"/>
       <c r="AK21" s="11"/>
-      <c r="AL21" s="46" t="s">
-        <v>40</v>
-      </c>
-      <c r="AM21" s="45"/>
-      <c r="AN21" s="45"/>
-      <c r="AO21" s="45"/>
+      <c r="AL21" s="37" t="s">
+        <v>44</v>
+      </c>
+      <c r="AM21" s="32"/>
+      <c r="AN21" s="32"/>
+      <c r="AO21" s="32"/>
       <c r="AP21" s="8"/>
     </row>
     <row r="22" spans="1:43" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -7844,22 +8697,7 @@
       <c r="AM1000" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="23">
-    <mergeCell ref="W13:AB13"/>
-    <mergeCell ref="AH13:AO13"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="I13:P13"/>
-    <mergeCell ref="N4:AD4"/>
-    <mergeCell ref="F4:M4"/>
-    <mergeCell ref="AL19:AO19"/>
-    <mergeCell ref="AL20:AO20"/>
-    <mergeCell ref="AL21:AO21"/>
-    <mergeCell ref="P20:W20"/>
-    <mergeCell ref="P21:W21"/>
+  <mergeCells count="22">
     <mergeCell ref="F21:K21"/>
     <mergeCell ref="AC21:AH21"/>
     <mergeCell ref="A19:B19"/>
@@ -7868,200 +8706,319 @@
     <mergeCell ref="AD19:AH19"/>
     <mergeCell ref="F20:K20"/>
     <mergeCell ref="AC20:AH20"/>
+    <mergeCell ref="AL19:AO19"/>
+    <mergeCell ref="AL20:AO20"/>
+    <mergeCell ref="AL21:AO21"/>
+    <mergeCell ref="P20:W20"/>
+    <mergeCell ref="P21:W21"/>
+    <mergeCell ref="W13:AB13"/>
+    <mergeCell ref="AH13:AO13"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="J4:AC4"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="I13:P13"/>
   </mergeCells>
-  <conditionalFormatting sqref="D9:E9">
-    <cfRule type="cellIs" dxfId="57" priority="61" operator="equal">
+  <conditionalFormatting sqref="Y9:Z9">
+    <cfRule type="cellIs" dxfId="177" priority="46" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="62" operator="equal">
+    <cfRule type="cellIs" dxfId="176" priority="47" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="55" priority="63" operator="equal">
+    <cfRule type="cellIs" dxfId="175" priority="48" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="64" operator="equal">
+    <cfRule type="cellIs" dxfId="174" priority="49" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="173" priority="50" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H9:I9">
+    <cfRule type="cellIs" dxfId="167" priority="26" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="166" priority="27" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="165" priority="28" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="164" priority="29" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="163" priority="30" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AG9">
+    <cfRule type="cellIs" dxfId="157" priority="41" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="156" priority="42" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="155" priority="43" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="154" priority="44" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="153" priority="45" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AF9:AG9">
+    <cfRule type="cellIs" dxfId="147" priority="36" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="146" priority="37" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="145" priority="38" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="144" priority="39" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="143" priority="40" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AC9:AE9">
+    <cfRule type="cellIs" dxfId="137" priority="31" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="136" priority="32" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="135" priority="33" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="134" priority="34" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="133" priority="35" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V9:W9">
+    <cfRule type="cellIs" dxfId="127" priority="16" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="126" priority="17" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="125" priority="18" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="124" priority="19" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="123" priority="20" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AC9:AD9">
+    <cfRule type="cellIs" dxfId="117" priority="11" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="116" priority="12" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="115" priority="13" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="114" priority="14" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="113" priority="15" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9">
+    <cfRule type="cellIs" dxfId="107" priority="6" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="106" priority="7" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="105" priority="8" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="104" priority="9" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="103" priority="10" operator="equal">
       <formula>7</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:AG10">
-    <cfRule type="cellIs" dxfId="53" priority="71" operator="equal">
+    <cfRule type="cellIs" dxfId="97" priority="71" operator="equal">
       <formula>"G"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="72" operator="equal">
+    <cfRule type="cellIs" dxfId="96" priority="72" operator="equal">
       <formula>"G"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="74" operator="equal">
+    <cfRule type="cellIs" dxfId="95" priority="73" operator="equal">
       <formula>"G"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="75" operator="equal">
+    <cfRule type="cellIs" dxfId="94" priority="74" operator="equal">
       <formula>"G"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="76" operator="equal">
+    <cfRule type="cellIs" dxfId="93" priority="75" operator="equal">
       <formula>"G"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="77" operator="equal">
+    <cfRule type="cellIs" dxfId="92" priority="76" operator="equal">
       <formula>"G"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="47" priority="78" operator="equal">
+    <cfRule type="cellIs" dxfId="91" priority="77" operator="equal">
       <formula>"G"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="79" operator="equal">
-      <formula>"G"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="80" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="81" operator="equal">
+    <cfRule type="cellIs" dxfId="90" priority="81" operator="equal">
       <formula>"L"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="82" operator="equal">
+    <cfRule type="cellIs" dxfId="89" priority="82" operator="equal">
       <formula>"L"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="83" operator="equal">
+    <cfRule type="cellIs" dxfId="88" priority="83" operator="equal">
       <formula>"L"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="41" priority="84" operator="equal">
+    <cfRule type="cellIs" dxfId="87" priority="84" operator="equal">
       <formula>"L"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="85" operator="equal">
+    <cfRule type="cellIs" dxfId="86" priority="85" operator="equal">
       <formula>"L"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="86" operator="equal">
+    <cfRule type="cellIs" dxfId="85" priority="86" operator="equal">
       <formula>"L"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="87" operator="equal">
+    <cfRule type="cellIs" dxfId="84" priority="87" operator="equal">
       <formula>"L"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="88" operator="equal">
+    <cfRule type="cellIs" dxfId="83" priority="88" operator="equal">
       <formula>"L"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="89" operator="equal">
+    <cfRule type="cellIs" dxfId="82" priority="89" operator="equal">
       <formula>"L"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G9:I9">
-    <cfRule type="cellIs" dxfId="35" priority="6" operator="equal">
+  <conditionalFormatting sqref="D7:AG10">
+    <cfRule type="cellIs" dxfId="65" priority="80" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="7" operator="equal">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D7:AG10">
+    <cfRule type="cellIs" dxfId="63" priority="78" operator="equal">
+      <formula>"G"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="62" priority="79" operator="equal">
+      <formula>"G"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA9:AB9">
+    <cfRule type="cellIs" dxfId="59" priority="66" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="58" priority="67" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="57" priority="68" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="56" priority="69" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="55" priority="70" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D9:E9">
+    <cfRule type="cellIs" dxfId="49" priority="61" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="48" priority="62" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="47" priority="63" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="46" priority="64" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="45" priority="65" operator="equal">
       <formula>7</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K9:L9">
-    <cfRule type="cellIs" dxfId="31" priority="56" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="56" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="57" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="57" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="29" priority="58" operator="equal">
+    <cfRule type="cellIs" dxfId="37" priority="58" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="59" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="59" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="35" priority="60" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R9:S9">
+    <cfRule type="cellIs" dxfId="29" priority="51" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="28" priority="52" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="27" priority="53" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="26" priority="54" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="25" priority="55" operator="equal">
       <formula>7</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O9:P9">
-    <cfRule type="cellIs" dxfId="27" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="21" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="22" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="23" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="23" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="24" operator="equal">
       <formula>7</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R9:S9">
-    <cfRule type="cellIs" dxfId="23" priority="51" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="52" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="53" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="54" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="25" operator="equal">
       <formula>7</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S9">
-    <cfRule type="cellIs" dxfId="19" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="2" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="4" operator="equal">
       <formula>7</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V9:W9">
-    <cfRule type="cellIs" dxfId="15" priority="16" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="17" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="18" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="19" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Y9:AG9">
-    <cfRule type="cellIs" dxfId="11" priority="31" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="32" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="33" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="34" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AC9:AD9">
-    <cfRule type="cellIs" dxfId="7" priority="11" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="12" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="13" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="14" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AG9">
-    <cfRule type="cellIs" dxfId="3" priority="41" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="42" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="43" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="44" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
       <formula>7</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Rebuild drivers timesheet tab with full feature set
- Add السائقين tab with name-based IDs, edit driver name, fill Fri (R)/Sat (Y)
- Fix day-1 import offset bug: drivers use col D (0-indexed=3), not col E (=4)
- Add built-in template export for drivers (public/templates/timesheet-drivers.xlsx, dayColStart=4)
- Restore TS_CODES_DRIVER, TAB_INFO drivers entry, and initial driver data in INITIAL_TS
- Bump storage key to boc_timesheet_v7 to avoid stale localStorage conflict
- Keep TimeSheetPage.js under 500 lines (499)
</commit_message>
<xml_diff>
--- a/public/templates/timesheet-drivers.xlsx
+++ b/public/templates/timesheet-drivers.xlsx
@@ -1,16 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ihab1980\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{661E4D9C-4826-449D-8BE1-0C8AB02B92DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1110" yWindow="570" windowWidth="18270" windowHeight="7110"/>
+    <workbookView xWindow="2190" yWindow="2355" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="الفاو " sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="Xn3YFQMmgadjBl8vW0I8rAQh3ekCSjPRpSw22WyK+vk="/>
     </ext>
@@ -168,7 +188,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -508,32 +528,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="14" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -543,7 +537,6 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -574,15 +567,57 @@
     <xf numFmtId="0" fontId="18" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
-  <dxfs count="184">
+  <dxfs count="58">
     <dxf>
       <fill>
         <patternFill patternType="lightGray"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="lightGrid"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid"/>
       </fill>
     </dxf>
     <dxf>
@@ -612,11 +647,6 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
         <patternFill patternType="gray125"/>
       </fill>
     </dxf>
@@ -628,11 +658,6 @@
     <dxf>
       <fill>
         <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
       </fill>
     </dxf>
     <dxf>
@@ -662,11 +687,6 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
         <patternFill patternType="gray125"/>
       </fill>
     </dxf>
@@ -678,11 +698,6 @@
     <dxf>
       <fill>
         <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
       </fill>
     </dxf>
     <dxf>
@@ -712,11 +727,6 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
         <patternFill patternType="gray125"/>
       </fill>
     </dxf>
@@ -728,11 +738,6 @@
     <dxf>
       <fill>
         <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
       </fill>
     </dxf>
     <dxf>
@@ -762,11 +767,6 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
         <patternFill patternType="gray125"/>
       </fill>
     </dxf>
@@ -778,148 +778,6 @@
     <dxf>
       <fill>
         <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid">
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid">
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
       </fill>
     </dxf>
     <dxf>
@@ -997,122 +855,21 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="3" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="lightGrid">
-          <bgColor theme="3" tint="0.79998168889431442"/>
+          <bgColor theme="9" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="lightGrid">
-          <fgColor theme="3" tint="0.59996337778862885"/>
-          <bgColor theme="3" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid">
-          <fgColor theme="3" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid">
-          <fgColor theme="3" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid">
-          <fgColor theme="3" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid">
-          <fgColor theme="3" tint="0.59996337778862885"/>
-          <bgColor theme="3" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="darkVertical">
-          <fgColor theme="0" tint="-0.14996795556505021"/>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightUp">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="darkHorizontal">
-          <fgColor theme="3" tint="0.59996337778862885"/>
-          <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightUp">
-          <fgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightUp">
-          <fgColor theme="5"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="darkTrellis">
-          <fgColor rgb="FFC00000"/>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="lightGrid">
-          <fgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1155,20 +912,8 @@
     <dxf>
       <fill>
         <patternFill patternType="lightGrid">
-          <fgColor theme="3" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid">
           <fgColor theme="3" tint="0.59996337778862885"/>
         </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
       </fill>
     </dxf>
     <dxf>
@@ -1191,446 +936,14 @@
         <patternFill patternType="solid"/>
       </fill>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGrid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE5B8B7"/>
-          <bgColor rgb="FFE5B8B7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE5B8B7"/>
-          <bgColor rgb="FFE5B8B7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1833,7 +1146,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AQ1000"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1854,13 +1167,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
@@ -1903,13 +1216,13 @@
       <c r="AQ1" s="7"/>
     </row>
     <row r="2" spans="1:43" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -2008,28 +1321,28 @@
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
       <c r="I4" s="7"/>
-      <c r="J4" s="35" t="s">
+      <c r="J4" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="K4" s="36"/>
-      <c r="L4" s="36"/>
-      <c r="M4" s="36"/>
-      <c r="N4" s="36"/>
-      <c r="O4" s="36"/>
-      <c r="P4" s="36"/>
-      <c r="Q4" s="36"/>
-      <c r="R4" s="36"/>
-      <c r="S4" s="36"/>
-      <c r="T4" s="36"/>
-      <c r="U4" s="36"/>
-      <c r="V4" s="36"/>
-      <c r="W4" s="36"/>
-      <c r="X4" s="36"/>
-      <c r="Y4" s="36"/>
-      <c r="Z4" s="36"/>
-      <c r="AA4" s="36"/>
-      <c r="AB4" s="36"/>
-      <c r="AC4" s="36"/>
+      <c r="K4" s="51"/>
+      <c r="L4" s="51"/>
+      <c r="M4" s="51"/>
+      <c r="N4" s="51"/>
+      <c r="O4" s="51"/>
+      <c r="P4" s="51"/>
+      <c r="Q4" s="51"/>
+      <c r="R4" s="51"/>
+      <c r="S4" s="51"/>
+      <c r="T4" s="51"/>
+      <c r="U4" s="51"/>
+      <c r="V4" s="51"/>
+      <c r="W4" s="51"/>
+      <c r="X4" s="51"/>
+      <c r="Y4" s="51"/>
+      <c r="Z4" s="51"/>
+      <c r="AA4" s="51"/>
+      <c r="AB4" s="51"/>
+      <c r="AC4" s="51"/>
       <c r="AD4" s="7"/>
       <c r="AE4" s="7"/>
       <c r="AF4" s="7"/>
@@ -2091,487 +1404,487 @@
       <c r="AQ5" s="7"/>
     </row>
     <row r="6" spans="1:43" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="50" t="s">
+      <c r="A6" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="51"/>
-      <c r="C6" s="52" t="s">
+      <c r="B6" s="40"/>
+      <c r="C6" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="53">
+      <c r="D6" s="42">
         <v>1</v>
       </c>
-      <c r="E6" s="53">
+      <c r="E6" s="42">
         <v>2</v>
       </c>
-      <c r="F6" s="53">
+      <c r="F6" s="42">
         <v>3</v>
       </c>
-      <c r="G6" s="53">
+      <c r="G6" s="42">
         <v>4</v>
       </c>
-      <c r="H6" s="53">
+      <c r="H6" s="42">
         <v>5</v>
       </c>
-      <c r="I6" s="53">
+      <c r="I6" s="42">
         <v>6</v>
       </c>
-      <c r="J6" s="53">
+      <c r="J6" s="42">
         <v>7</v>
       </c>
-      <c r="K6" s="53">
+      <c r="K6" s="42">
         <v>8</v>
       </c>
-      <c r="L6" s="53">
+      <c r="L6" s="42">
         <v>9</v>
       </c>
-      <c r="M6" s="53">
+      <c r="M6" s="42">
         <v>10</v>
       </c>
-      <c r="N6" s="53">
+      <c r="N6" s="42">
         <v>11</v>
       </c>
-      <c r="O6" s="53">
+      <c r="O6" s="42">
         <v>12</v>
       </c>
-      <c r="P6" s="53">
+      <c r="P6" s="42">
         <v>13</v>
       </c>
-      <c r="Q6" s="53">
+      <c r="Q6" s="42">
         <v>14</v>
       </c>
-      <c r="R6" s="53">
+      <c r="R6" s="42">
         <v>15</v>
       </c>
-      <c r="S6" s="53">
+      <c r="S6" s="42">
         <v>16</v>
       </c>
-      <c r="T6" s="53">
+      <c r="T6" s="42">
         <v>17</v>
       </c>
-      <c r="U6" s="53">
+      <c r="U6" s="42">
         <v>18</v>
       </c>
-      <c r="V6" s="53">
+      <c r="V6" s="42">
         <v>19</v>
       </c>
-      <c r="W6" s="53">
+      <c r="W6" s="42">
         <v>20</v>
       </c>
-      <c r="X6" s="53">
+      <c r="X6" s="42">
         <v>21</v>
       </c>
-      <c r="Y6" s="53">
+      <c r="Y6" s="42">
         <v>22</v>
       </c>
-      <c r="Z6" s="53">
+      <c r="Z6" s="42">
         <v>23</v>
       </c>
-      <c r="AA6" s="53">
+      <c r="AA6" s="42">
         <v>24</v>
       </c>
-      <c r="AB6" s="53">
+      <c r="AB6" s="42">
         <v>25</v>
       </c>
-      <c r="AC6" s="53">
+      <c r="AC6" s="42">
         <v>26</v>
       </c>
-      <c r="AD6" s="53">
+      <c r="AD6" s="42">
         <v>27</v>
       </c>
-      <c r="AE6" s="53">
+      <c r="AE6" s="42">
         <v>28</v>
       </c>
-      <c r="AF6" s="53">
+      <c r="AF6" s="42">
         <v>29</v>
       </c>
-      <c r="AG6" s="53">
+      <c r="AG6" s="42">
         <v>30</v>
       </c>
-      <c r="AH6" s="52" t="s">
+      <c r="AH6" s="41" t="s">
         <v>7</v>
       </c>
-      <c r="AI6" s="52" t="s">
+      <c r="AI6" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="AJ6" s="50" t="s">
+      <c r="AJ6" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="AK6" s="50" t="s">
+      <c r="AK6" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="AL6" s="54" t="s">
+      <c r="AL6" s="43" t="s">
         <v>11</v>
       </c>
-      <c r="AM6" s="54" t="s">
+      <c r="AM6" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="AN6" s="54" t="s">
+      <c r="AN6" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="AO6" s="54" t="s">
+      <c r="AO6" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="AP6" s="54" t="s">
+      <c r="AP6" s="43" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:43" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="39" t="s">
+      <c r="A7" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="40"/>
-      <c r="C7" s="41" t="s">
+      <c r="B7" s="54"/>
+      <c r="C7" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="48" t="s">
+      <c r="D7" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="48"/>
-      <c r="F7" s="48" t="s">
+      <c r="E7" s="37"/>
+      <c r="F7" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="G7" s="49" t="s">
+      <c r="G7" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="H7" s="49" t="s">
+      <c r="H7" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="I7" s="49" t="s">
+      <c r="I7" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="J7" s="48" t="s">
+      <c r="J7" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="K7" s="48" t="s">
+      <c r="K7" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="L7" s="48" t="s">
+      <c r="L7" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="M7" s="48" t="s">
+      <c r="M7" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="N7" s="48" t="s">
+      <c r="N7" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="O7" s="49" t="s">
+      <c r="O7" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="P7" s="49" t="s">
+      <c r="P7" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="Q7" s="48" t="s">
+      <c r="Q7" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="R7" s="48" t="s">
+      <c r="R7" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="S7" s="49" t="s">
+      <c r="S7" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="T7" s="48" t="s">
+      <c r="T7" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="U7" s="48" t="s">
+      <c r="U7" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="V7" s="49" t="s">
+      <c r="V7" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="W7" s="49" t="s">
+      <c r="W7" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="X7" s="48" t="s">
+      <c r="X7" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="Y7" s="48" t="s">
+      <c r="Y7" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="Z7" s="48" t="s">
+      <c r="Z7" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="AA7" s="48"/>
-      <c r="AB7" s="48"/>
-      <c r="AC7" s="49" t="s">
+      <c r="AA7" s="37"/>
+      <c r="AB7" s="37"/>
+      <c r="AC7" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="AD7" s="49" t="s">
+      <c r="AD7" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="AE7" s="48"/>
-      <c r="AF7" s="48"/>
-      <c r="AG7" s="48"/>
-      <c r="AH7" s="42"/>
-      <c r="AI7" s="42">
+      <c r="AE7" s="37"/>
+      <c r="AF7" s="37"/>
+      <c r="AG7" s="37"/>
+      <c r="AH7" s="32"/>
+      <c r="AI7" s="32">
         <f>COUNTIF(D7:AG7,"ف")</f>
         <v>0</v>
       </c>
-      <c r="AJ7" s="43">
+      <c r="AJ7" s="33">
         <f>COUNTIF(D7:AG7,"أ")</f>
         <v>0</v>
       </c>
-      <c r="AK7" s="43">
+      <c r="AK7" s="33">
         <f>COUNTIF(D7:AG7,"ب")</f>
         <v>0</v>
       </c>
-      <c r="AL7" s="43">
+      <c r="AL7" s="33">
         <f t="shared" ref="AL7:AL10" si="0">COUNTIF(D7:AH7,"ر")</f>
         <v>0</v>
       </c>
-      <c r="AM7" s="43">
+      <c r="AM7" s="33">
         <f>COUNTIF(D7:AG7,"ق")</f>
         <v>1</v>
       </c>
-      <c r="AN7" s="43">
+      <c r="AN7" s="33">
         <f>COUNTIF(G7:AI7,"Y")</f>
         <v>6</v>
       </c>
-      <c r="AO7" s="43"/>
-      <c r="AP7" s="43"/>
+      <c r="AO7" s="33"/>
+      <c r="AP7" s="33"/>
       <c r="AQ7" s="10"/>
     </row>
     <row r="8" spans="1:43" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="44"/>
-      <c r="B8" s="44"/>
-      <c r="C8" s="45" t="s">
+      <c r="A8" s="53"/>
+      <c r="B8" s="53"/>
+      <c r="C8" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="48"/>
-      <c r="E8" s="48"/>
-      <c r="F8" s="48"/>
-      <c r="G8" s="49"/>
-      <c r="H8" s="49"/>
-      <c r="I8" s="49"/>
-      <c r="J8" s="48"/>
-      <c r="K8" s="48"/>
-      <c r="L8" s="48"/>
-      <c r="M8" s="48"/>
-      <c r="N8" s="48"/>
-      <c r="O8" s="49"/>
-      <c r="P8" s="49"/>
-      <c r="Q8" s="48"/>
-      <c r="R8" s="48"/>
-      <c r="S8" s="49"/>
-      <c r="T8" s="48"/>
-      <c r="U8" s="48"/>
-      <c r="V8" s="49"/>
-      <c r="W8" s="49"/>
-      <c r="X8" s="48"/>
-      <c r="Y8" s="48"/>
-      <c r="Z8" s="48"/>
-      <c r="AA8" s="48"/>
-      <c r="AB8" s="48"/>
-      <c r="AC8" s="49"/>
-      <c r="AD8" s="49"/>
-      <c r="AE8" s="48"/>
-      <c r="AF8" s="48"/>
-      <c r="AG8" s="48"/>
-      <c r="AH8" s="46">
+      <c r="D8" s="37"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="38"/>
+      <c r="I8" s="38"/>
+      <c r="J8" s="37"/>
+      <c r="K8" s="37"/>
+      <c r="L8" s="37"/>
+      <c r="M8" s="37"/>
+      <c r="N8" s="37"/>
+      <c r="O8" s="38"/>
+      <c r="P8" s="38"/>
+      <c r="Q8" s="37"/>
+      <c r="R8" s="37"/>
+      <c r="S8" s="38"/>
+      <c r="T8" s="37"/>
+      <c r="U8" s="37"/>
+      <c r="V8" s="38"/>
+      <c r="W8" s="38"/>
+      <c r="X8" s="37"/>
+      <c r="Y8" s="37"/>
+      <c r="Z8" s="37"/>
+      <c r="AA8" s="37"/>
+      <c r="AB8" s="37"/>
+      <c r="AC8" s="38"/>
+      <c r="AD8" s="38"/>
+      <c r="AE8" s="37"/>
+      <c r="AF8" s="37"/>
+      <c r="AG8" s="37"/>
+      <c r="AH8" s="35">
         <f>SUM(D8:AG8)</f>
         <v>0</v>
       </c>
-      <c r="AI8" s="42">
+      <c r="AI8" s="32">
         <f>COUNTIF(D8:AG8,"ف")</f>
         <v>0</v>
       </c>
-      <c r="AJ8" s="43">
+      <c r="AJ8" s="33">
         <f>COUNTIF(D8:AG8,"أ")</f>
         <v>0</v>
       </c>
-      <c r="AK8" s="43">
+      <c r="AK8" s="33">
         <v>0</v>
       </c>
-      <c r="AL8" s="43">
+      <c r="AL8" s="33">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="AM8" s="43">
+      <c r="AM8" s="33">
         <v>0</v>
       </c>
-      <c r="AN8" s="43"/>
-      <c r="AO8" s="43"/>
-      <c r="AP8" s="43"/>
+      <c r="AN8" s="33"/>
+      <c r="AO8" s="33"/>
+      <c r="AP8" s="33"/>
       <c r="AQ8" s="10"/>
     </row>
     <row r="9" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="43" t="s">
+      <c r="A9" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="47"/>
-      <c r="C9" s="41" t="s">
+      <c r="B9" s="36"/>
+      <c r="C9" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="48" t="s">
+      <c r="D9" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="E9" s="48" t="s">
+      <c r="E9" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="F9" s="48" t="s">
+      <c r="F9" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="G9" s="49" t="s">
+      <c r="G9" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="H9" s="49" t="s">
+      <c r="H9" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="I9" s="49" t="s">
+      <c r="I9" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="J9" s="48" t="s">
+      <c r="J9" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="K9" s="48" t="s">
+      <c r="K9" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="L9" s="48" t="s">
+      <c r="L9" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="M9" s="48" t="s">
+      <c r="M9" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="N9" s="48" t="s">
+      <c r="N9" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="O9" s="49" t="s">
+      <c r="O9" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="P9" s="49" t="s">
+      <c r="P9" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="Q9" s="48" t="s">
+      <c r="Q9" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="R9" s="48" t="s">
+      <c r="R9" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="S9" s="49" t="s">
+      <c r="S9" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="T9" s="48" t="s">
+      <c r="T9" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="U9" s="48" t="s">
+      <c r="U9" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="V9" s="49" t="s">
+      <c r="V9" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="W9" s="49" t="s">
+      <c r="W9" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="X9" s="48" t="s">
+      <c r="X9" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="Y9" s="48" t="s">
+      <c r="Y9" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="Z9" s="48" t="s">
+      <c r="Z9" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="AA9" s="48"/>
-      <c r="AB9" s="48"/>
-      <c r="AC9" s="49" t="s">
+      <c r="AA9" s="37"/>
+      <c r="AB9" s="37"/>
+      <c r="AC9" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="AD9" s="49" t="s">
+      <c r="AD9" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="AE9" s="48"/>
-      <c r="AF9" s="48"/>
-      <c r="AG9" s="48"/>
-      <c r="AH9" s="42"/>
-      <c r="AI9" s="42">
+      <c r="AE9" s="37"/>
+      <c r="AF9" s="37"/>
+      <c r="AG9" s="37"/>
+      <c r="AH9" s="32"/>
+      <c r="AI9" s="32">
         <f>COUNTIF(D9:AG9,"ف")</f>
         <v>0</v>
       </c>
-      <c r="AJ9" s="43">
+      <c r="AJ9" s="33">
         <f>COUNTIF(D9:AG9,"أ")</f>
         <v>0</v>
       </c>
-      <c r="AK9" s="43">
+      <c r="AK9" s="33">
         <f>COUNTIF(D7:AG7,"ب")</f>
         <v>0</v>
       </c>
-      <c r="AL9" s="43">
+      <c r="AL9" s="33">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="AM9" s="43">
+      <c r="AM9" s="33">
         <f>COUNTIF(D7:AG7,"ق")</f>
         <v>1</v>
       </c>
-      <c r="AN9" s="43"/>
-      <c r="AO9" s="43"/>
-      <c r="AP9" s="43"/>
+      <c r="AN9" s="33"/>
+      <c r="AO9" s="33"/>
+      <c r="AP9" s="33"/>
       <c r="AQ9" s="10"/>
     </row>
     <row r="10" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="47"/>
-      <c r="B10" s="47"/>
-      <c r="C10" s="45" t="s">
+      <c r="A10" s="36"/>
+      <c r="B10" s="36"/>
+      <c r="C10" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="48"/>
-      <c r="E10" s="48"/>
-      <c r="F10" s="48"/>
-      <c r="G10" s="49"/>
-      <c r="H10" s="49"/>
-      <c r="I10" s="49"/>
-      <c r="J10" s="48"/>
-      <c r="K10" s="48"/>
-      <c r="L10" s="48"/>
-      <c r="M10" s="48"/>
-      <c r="N10" s="48"/>
-      <c r="O10" s="49"/>
-      <c r="P10" s="49"/>
-      <c r="Q10" s="48"/>
-      <c r="R10" s="48"/>
-      <c r="S10" s="49"/>
-      <c r="T10" s="48"/>
-      <c r="U10" s="48"/>
-      <c r="V10" s="49"/>
-      <c r="W10" s="49"/>
-      <c r="X10" s="48"/>
-      <c r="Y10" s="48"/>
-      <c r="Z10" s="48"/>
-      <c r="AA10" s="48"/>
-      <c r="AB10" s="48"/>
-      <c r="AC10" s="49"/>
-      <c r="AD10" s="49"/>
-      <c r="AE10" s="48"/>
-      <c r="AF10" s="48"/>
-      <c r="AG10" s="48"/>
-      <c r="AH10" s="46">
+      <c r="D10" s="37"/>
+      <c r="E10" s="37"/>
+      <c r="F10" s="37"/>
+      <c r="G10" s="38"/>
+      <c r="H10" s="38"/>
+      <c r="I10" s="38"/>
+      <c r="J10" s="37"/>
+      <c r="K10" s="37"/>
+      <c r="L10" s="37"/>
+      <c r="M10" s="37"/>
+      <c r="N10" s="37"/>
+      <c r="O10" s="38"/>
+      <c r="P10" s="38"/>
+      <c r="Q10" s="37"/>
+      <c r="R10" s="37"/>
+      <c r="S10" s="38"/>
+      <c r="T10" s="37"/>
+      <c r="U10" s="37"/>
+      <c r="V10" s="38"/>
+      <c r="W10" s="38"/>
+      <c r="X10" s="37"/>
+      <c r="Y10" s="37"/>
+      <c r="Z10" s="37"/>
+      <c r="AA10" s="37"/>
+      <c r="AB10" s="37"/>
+      <c r="AC10" s="38"/>
+      <c r="AD10" s="38"/>
+      <c r="AE10" s="37"/>
+      <c r="AF10" s="37"/>
+      <c r="AG10" s="37"/>
+      <c r="AH10" s="35">
         <f>SUM(D10:AG10)</f>
         <v>0</v>
       </c>
-      <c r="AI10" s="42">
+      <c r="AI10" s="32">
         <f>COUNTIF(D10:AG10,"ف")</f>
         <v>0</v>
       </c>
-      <c r="AJ10" s="42">
+      <c r="AJ10" s="32">
         <f>COUNTIF(D10:AG10,"أ")</f>
         <v>0</v>
       </c>
-      <c r="AK10" s="42">
+      <c r="AK10" s="32">
         <f>COUNTIF(D10:AG10,"ب")</f>
         <v>0</v>
       </c>
-      <c r="AL10" s="42">
+      <c r="AL10" s="32">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="AM10" s="42">
+      <c r="AM10" s="32">
         <v>0</v>
       </c>
-      <c r="AN10" s="42">
+      <c r="AN10" s="32">
         <v>0</v>
       </c>
-      <c r="AO10" s="43"/>
-      <c r="AP10" s="43"/>
+      <c r="AO10" s="33"/>
+      <c r="AP10" s="33"/>
       <c r="AQ10" s="10"/>
     </row>
     <row r="11" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2630,55 +1943,55 @@
       <c r="AQ12" s="8"/>
     </row>
     <row r="13" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="31" t="s">
+      <c r="A13" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="32"/>
+      <c r="B13" s="45"/>
       <c r="C13" s="15"/>
       <c r="D13" s="16"/>
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
       <c r="G13" s="16"/>
       <c r="H13" s="15"/>
-      <c r="I13" s="31" t="s">
+      <c r="I13" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="J13" s="32"/>
-      <c r="K13" s="32"/>
-      <c r="L13" s="32"/>
-      <c r="M13" s="32"/>
-      <c r="N13" s="32"/>
-      <c r="O13" s="32"/>
-      <c r="P13" s="32"/>
+      <c r="J13" s="45"/>
+      <c r="K13" s="45"/>
+      <c r="L13" s="45"/>
+      <c r="M13" s="45"/>
+      <c r="N13" s="45"/>
+      <c r="O13" s="45"/>
+      <c r="P13" s="45"/>
       <c r="Q13" s="16"/>
       <c r="R13" s="16"/>
       <c r="S13" s="16"/>
       <c r="T13" s="16"/>
       <c r="U13" s="16"/>
       <c r="V13" s="16"/>
-      <c r="W13" s="31" t="s">
+      <c r="W13" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="X13" s="32"/>
-      <c r="Y13" s="32"/>
-      <c r="Z13" s="32"/>
-      <c r="AA13" s="32"/>
-      <c r="AB13" s="32"/>
+      <c r="X13" s="45"/>
+      <c r="Y13" s="45"/>
+      <c r="Z13" s="45"/>
+      <c r="AA13" s="45"/>
+      <c r="AB13" s="45"/>
       <c r="AC13" s="15"/>
       <c r="AD13" s="15"/>
       <c r="AE13" s="15"/>
       <c r="AF13" s="15"/>
       <c r="AG13" s="15"/>
-      <c r="AH13" s="33" t="s">
+      <c r="AH13" s="48" t="s">
         <v>28</v>
       </c>
-      <c r="AI13" s="32"/>
-      <c r="AJ13" s="32"/>
-      <c r="AK13" s="32"/>
-      <c r="AL13" s="32"/>
-      <c r="AM13" s="32"/>
-      <c r="AN13" s="32"/>
-      <c r="AO13" s="32"/>
+      <c r="AI13" s="45"/>
+      <c r="AJ13" s="45"/>
+      <c r="AK13" s="45"/>
+      <c r="AL13" s="45"/>
+      <c r="AM13" s="45"/>
+      <c r="AN13" s="45"/>
+      <c r="AO13" s="45"/>
       <c r="AP13" s="17" t="s">
         <v>29</v>
       </c>
@@ -2920,57 +2233,57 @@
       <c r="AQ18" s="8"/>
     </row>
     <row r="19" spans="1:43" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="37" t="s">
+      <c r="A19" s="46" t="s">
         <v>35</v>
       </c>
-      <c r="B19" s="32"/>
+      <c r="B19" s="45"/>
       <c r="C19" s="25"/>
       <c r="D19" s="26"/>
-      <c r="E19" s="37" t="s">
+      <c r="E19" s="46" t="s">
         <v>36</v>
       </c>
-      <c r="F19" s="32"/>
-      <c r="G19" s="32"/>
-      <c r="H19" s="32"/>
-      <c r="I19" s="32"/>
-      <c r="J19" s="32"/>
-      <c r="K19" s="32"/>
-      <c r="L19" s="32"/>
+      <c r="F19" s="45"/>
+      <c r="G19" s="45"/>
+      <c r="H19" s="45"/>
+      <c r="I19" s="45"/>
+      <c r="J19" s="45"/>
+      <c r="K19" s="45"/>
+      <c r="L19" s="45"/>
       <c r="M19" s="27"/>
       <c r="N19" s="26"/>
       <c r="O19" s="26"/>
-      <c r="P19" s="37" t="s">
+      <c r="P19" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="Q19" s="32"/>
-      <c r="R19" s="32"/>
-      <c r="S19" s="32"/>
-      <c r="T19" s="32"/>
-      <c r="U19" s="32"/>
-      <c r="V19" s="32"/>
-      <c r="W19" s="32"/>
-      <c r="X19" s="32"/>
-      <c r="Y19" s="32"/>
+      <c r="Q19" s="45"/>
+      <c r="R19" s="45"/>
+      <c r="S19" s="45"/>
+      <c r="T19" s="45"/>
+      <c r="U19" s="45"/>
+      <c r="V19" s="45"/>
+      <c r="W19" s="45"/>
+      <c r="X19" s="45"/>
+      <c r="Y19" s="45"/>
       <c r="Z19" s="26"/>
       <c r="AA19" s="26"/>
       <c r="AB19" s="26"/>
       <c r="AC19" s="25"/>
-      <c r="AD19" s="37" t="s">
+      <c r="AD19" s="46" t="s">
         <v>38</v>
       </c>
-      <c r="AE19" s="32"/>
-      <c r="AF19" s="32"/>
-      <c r="AG19" s="32"/>
-      <c r="AH19" s="32"/>
+      <c r="AE19" s="45"/>
+      <c r="AF19" s="45"/>
+      <c r="AG19" s="45"/>
+      <c r="AH19" s="45"/>
       <c r="AI19" s="26"/>
       <c r="AJ19" s="11"/>
       <c r="AK19" s="11"/>
-      <c r="AL19" s="37" t="s">
+      <c r="AL19" s="46" t="s">
         <v>39</v>
       </c>
-      <c r="AM19" s="32"/>
-      <c r="AN19" s="32"/>
-      <c r="AO19" s="32"/>
+      <c r="AM19" s="45"/>
+      <c r="AN19" s="45"/>
+      <c r="AO19" s="45"/>
       <c r="AP19" s="24" t="s">
         <v>40</v>
       </c>
@@ -2982,46 +2295,46 @@
       <c r="C20" s="26"/>
       <c r="D20" s="26"/>
       <c r="E20" s="26"/>
-      <c r="F20" s="38"/>
-      <c r="G20" s="32"/>
-      <c r="H20" s="32"/>
-      <c r="I20" s="32"/>
-      <c r="J20" s="32"/>
-      <c r="K20" s="32"/>
+      <c r="F20" s="44"/>
+      <c r="G20" s="45"/>
+      <c r="H20" s="45"/>
+      <c r="I20" s="45"/>
+      <c r="J20" s="45"/>
+      <c r="K20" s="45"/>
       <c r="L20" s="26"/>
       <c r="M20" s="27"/>
       <c r="N20" s="26"/>
       <c r="O20" s="26"/>
-      <c r="P20" s="38"/>
-      <c r="Q20" s="32"/>
-      <c r="R20" s="32"/>
-      <c r="S20" s="32"/>
-      <c r="T20" s="32"/>
-      <c r="U20" s="32"/>
-      <c r="V20" s="32"/>
-      <c r="W20" s="32"/>
+      <c r="P20" s="44"/>
+      <c r="Q20" s="45"/>
+      <c r="R20" s="45"/>
+      <c r="S20" s="45"/>
+      <c r="T20" s="45"/>
+      <c r="U20" s="45"/>
+      <c r="V20" s="45"/>
+      <c r="W20" s="45"/>
       <c r="X20" s="26"/>
       <c r="Y20" s="26"/>
       <c r="Z20" s="26"/>
       <c r="AA20" s="26"/>
       <c r="AB20" s="26"/>
-      <c r="AC20" s="37" t="s">
+      <c r="AC20" s="46" t="s">
         <v>41</v>
       </c>
-      <c r="AD20" s="32"/>
-      <c r="AE20" s="32"/>
-      <c r="AF20" s="32"/>
-      <c r="AG20" s="32"/>
-      <c r="AH20" s="32"/>
+      <c r="AD20" s="45"/>
+      <c r="AE20" s="45"/>
+      <c r="AF20" s="45"/>
+      <c r="AG20" s="45"/>
+      <c r="AH20" s="45"/>
       <c r="AI20" s="26"/>
       <c r="AJ20" s="11"/>
       <c r="AK20" s="11"/>
-      <c r="AL20" s="37" t="s">
+      <c r="AL20" s="46" t="s">
         <v>42</v>
       </c>
-      <c r="AM20" s="32"/>
-      <c r="AN20" s="32"/>
-      <c r="AO20" s="32"/>
+      <c r="AM20" s="45"/>
+      <c r="AN20" s="45"/>
+      <c r="AO20" s="45"/>
       <c r="AP20" s="8"/>
       <c r="AQ20" s="8"/>
     </row>
@@ -3031,46 +2344,46 @@
       <c r="C21" s="26"/>
       <c r="D21" s="26"/>
       <c r="E21" s="26"/>
-      <c r="F21" s="38"/>
-      <c r="G21" s="32"/>
-      <c r="H21" s="32"/>
-      <c r="I21" s="32"/>
-      <c r="J21" s="32"/>
-      <c r="K21" s="32"/>
+      <c r="F21" s="44"/>
+      <c r="G21" s="45"/>
+      <c r="H21" s="45"/>
+      <c r="I21" s="45"/>
+      <c r="J21" s="45"/>
+      <c r="K21" s="45"/>
       <c r="L21" s="26"/>
       <c r="M21" s="27"/>
       <c r="N21" s="26"/>
       <c r="O21" s="26"/>
-      <c r="P21" s="38"/>
-      <c r="Q21" s="32"/>
-      <c r="R21" s="32"/>
-      <c r="S21" s="32"/>
-      <c r="T21" s="32"/>
-      <c r="U21" s="32"/>
-      <c r="V21" s="32"/>
-      <c r="W21" s="32"/>
+      <c r="P21" s="44"/>
+      <c r="Q21" s="45"/>
+      <c r="R21" s="45"/>
+      <c r="S21" s="45"/>
+      <c r="T21" s="45"/>
+      <c r="U21" s="45"/>
+      <c r="V21" s="45"/>
+      <c r="W21" s="45"/>
       <c r="X21" s="26"/>
       <c r="Y21" s="26"/>
       <c r="Z21" s="26"/>
       <c r="AA21" s="26"/>
       <c r="AB21" s="26"/>
-      <c r="AC21" s="37" t="s">
+      <c r="AC21" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="AD21" s="32"/>
-      <c r="AE21" s="32"/>
-      <c r="AF21" s="32"/>
-      <c r="AG21" s="32"/>
-      <c r="AH21" s="32"/>
+      <c r="AD21" s="45"/>
+      <c r="AE21" s="45"/>
+      <c r="AF21" s="45"/>
+      <c r="AG21" s="45"/>
+      <c r="AH21" s="45"/>
       <c r="AI21" s="26"/>
       <c r="AJ21" s="11"/>
       <c r="AK21" s="11"/>
-      <c r="AL21" s="37" t="s">
+      <c r="AL21" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="AM21" s="32"/>
-      <c r="AN21" s="32"/>
-      <c r="AO21" s="32"/>
+      <c r="AM21" s="45"/>
+      <c r="AN21" s="45"/>
+      <c r="AO21" s="45"/>
       <c r="AP21" s="8"/>
     </row>
     <row r="22" spans="1:43" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -8698,19 +8011,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="F21:K21"/>
-    <mergeCell ref="AC21:AH21"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="E19:L19"/>
-    <mergeCell ref="P19:Y19"/>
-    <mergeCell ref="AD19:AH19"/>
-    <mergeCell ref="F20:K20"/>
-    <mergeCell ref="AC20:AH20"/>
-    <mergeCell ref="AL19:AO19"/>
-    <mergeCell ref="AL20:AO20"/>
-    <mergeCell ref="AL21:AO21"/>
-    <mergeCell ref="P20:W20"/>
-    <mergeCell ref="P21:W21"/>
     <mergeCell ref="W13:AB13"/>
     <mergeCell ref="AH13:AO13"/>
     <mergeCell ref="A1:E1"/>
@@ -8720,305 +8020,213 @@
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="I13:P13"/>
+    <mergeCell ref="AL19:AO19"/>
+    <mergeCell ref="AL20:AO20"/>
+    <mergeCell ref="AL21:AO21"/>
+    <mergeCell ref="P20:W20"/>
+    <mergeCell ref="P21:W21"/>
+    <mergeCell ref="F21:K21"/>
+    <mergeCell ref="AC21:AH21"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="E19:L19"/>
+    <mergeCell ref="P19:Y19"/>
+    <mergeCell ref="AD19:AH19"/>
+    <mergeCell ref="F20:K20"/>
+    <mergeCell ref="AC20:AH20"/>
   </mergeCells>
-  <conditionalFormatting sqref="Y9:Z9">
-    <cfRule type="cellIs" dxfId="177" priority="46" operator="equal">
+  <conditionalFormatting sqref="D9:E9">
+    <cfRule type="cellIs" dxfId="57" priority="61" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="176" priority="47" operator="equal">
+    <cfRule type="cellIs" dxfId="56" priority="62" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="175" priority="48" operator="equal">
+    <cfRule type="cellIs" dxfId="55" priority="63" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="174" priority="49" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="173" priority="50" operator="equal">
+    <cfRule type="cellIs" dxfId="54" priority="64" operator="equal">
       <formula>7</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:I9">
-    <cfRule type="cellIs" dxfId="167" priority="26" operator="equal">
+  <conditionalFormatting sqref="D7:AG10">
+    <cfRule type="cellIs" dxfId="53" priority="71" operator="equal">
+      <formula>"G"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="52" priority="72" operator="equal">
+      <formula>"G"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="51" priority="74" operator="equal">
+      <formula>"G"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="50" priority="75" operator="equal">
+      <formula>"G"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="49" priority="76" operator="equal">
+      <formula>"G"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="48" priority="77" operator="equal">
+      <formula>"G"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="47" priority="78" operator="equal">
+      <formula>"G"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="46" priority="79" operator="equal">
+      <formula>"G"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="45" priority="80" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="166" priority="27" operator="equal">
+    <cfRule type="cellIs" dxfId="44" priority="81" operator="equal">
+      <formula>"L"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="43" priority="82" operator="equal">
+      <formula>"L"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="42" priority="83" operator="equal">
+      <formula>"L"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="41" priority="84" operator="equal">
+      <formula>"L"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="40" priority="85" operator="equal">
+      <formula>"L"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="39" priority="86" operator="equal">
+      <formula>"L"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="38" priority="87" operator="equal">
+      <formula>"L"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="37" priority="88" operator="equal">
+      <formula>"L"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="36" priority="89" operator="equal">
+      <formula>"L"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9:I9">
+    <cfRule type="cellIs" dxfId="35" priority="6" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="165" priority="28" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="7" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="164" priority="29" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="8" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="163" priority="30" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="9" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K9:L9">
+    <cfRule type="cellIs" dxfId="31" priority="56" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="30" priority="57" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="29" priority="58" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="28" priority="59" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O9:P9">
+    <cfRule type="cellIs" dxfId="27" priority="21" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="26" priority="22" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="25" priority="23" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="24" priority="24" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R9:S9">
+    <cfRule type="cellIs" dxfId="23" priority="51" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="22" priority="52" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="21" priority="53" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="20" priority="54" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S9">
+    <cfRule type="cellIs" dxfId="19" priority="1" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="18" priority="2" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="17" priority="3" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="16" priority="4" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V9:W9">
+    <cfRule type="cellIs" dxfId="15" priority="16" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="14" priority="17" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="13" priority="18" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="19" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Y9:AG9">
+    <cfRule type="cellIs" dxfId="11" priority="31" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="32" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="33" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="34" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AC9:AD9">
+    <cfRule type="cellIs" dxfId="7" priority="11" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="12" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="13" operator="equal">
+      <formula>7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="14" operator="equal">
       <formula>7</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AG9">
-    <cfRule type="cellIs" dxfId="157" priority="41" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="41" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="156" priority="42" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="42" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="155" priority="43" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="43" operator="equal">
       <formula>7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="154" priority="44" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="153" priority="45" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AF9:AG9">
-    <cfRule type="cellIs" dxfId="147" priority="36" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="146" priority="37" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="145" priority="38" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="144" priority="39" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="143" priority="40" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AC9:AE9">
-    <cfRule type="cellIs" dxfId="137" priority="31" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="136" priority="32" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="135" priority="33" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="134" priority="34" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="133" priority="35" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V9:W9">
-    <cfRule type="cellIs" dxfId="127" priority="16" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="126" priority="17" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="125" priority="18" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="124" priority="19" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="123" priority="20" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AC9:AD9">
-    <cfRule type="cellIs" dxfId="117" priority="11" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="116" priority="12" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="115" priority="13" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="114" priority="14" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="113" priority="15" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G9">
-    <cfRule type="cellIs" dxfId="107" priority="6" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="106" priority="7" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="105" priority="8" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="104" priority="9" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="103" priority="10" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D7:AG10">
-    <cfRule type="cellIs" dxfId="97" priority="71" operator="equal">
-      <formula>"G"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="96" priority="72" operator="equal">
-      <formula>"G"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="95" priority="73" operator="equal">
-      <formula>"G"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="94" priority="74" operator="equal">
-      <formula>"G"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="93" priority="75" operator="equal">
-      <formula>"G"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="92" priority="76" operator="equal">
-      <formula>"G"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="91" priority="77" operator="equal">
-      <formula>"G"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="90" priority="81" operator="equal">
-      <formula>"L"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="89" priority="82" operator="equal">
-      <formula>"L"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="88" priority="83" operator="equal">
-      <formula>"L"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="87" priority="84" operator="equal">
-      <formula>"L"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="86" priority="85" operator="equal">
-      <formula>"L"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="85" priority="86" operator="equal">
-      <formula>"L"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="84" priority="87" operator="equal">
-      <formula>"L"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="83" priority="88" operator="equal">
-      <formula>"L"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="82" priority="89" operator="equal">
-      <formula>"L"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D7:AG10">
-    <cfRule type="cellIs" dxfId="65" priority="80" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D7:AG10">
-    <cfRule type="cellIs" dxfId="63" priority="78" operator="equal">
-      <formula>"G"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="62" priority="79" operator="equal">
-      <formula>"G"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AA9:AB9">
-    <cfRule type="cellIs" dxfId="59" priority="66" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="67" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="57" priority="68" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="69" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="55" priority="70" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D9:E9">
-    <cfRule type="cellIs" dxfId="49" priority="61" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="62" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="47" priority="63" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="64" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="65" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K9:L9">
-    <cfRule type="cellIs" dxfId="39" priority="56" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="57" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="58" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="59" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="35" priority="60" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R9:S9">
-    <cfRule type="cellIs" dxfId="29" priority="51" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="52" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="53" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="54" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="55" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O9:P9">
-    <cfRule type="cellIs" dxfId="19" priority="21" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="22" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="23" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="24" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="25" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S9">
-    <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="2" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="4" operator="equal">
-      <formula>7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="44" operator="equal">
       <formula>7</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>